<commit_message>
Add Clown Shoes and Crown items with perfect-game and level-up systems
- ItemData: perfect_aware/perfect_effects/perfect_save_chance for
  perfect-game tracking, and bonus_level_up_chance for Crown-style
  extra level-ups.
- CharacterData: structured level_up_stats + level_up_reward_type/amount.
- GameState: player_level + last_game_perfected (saved/reset), and
  apply_level_up_stats() to fold a character's level-up stat block in.
- Overworld verification modal: shows a Perfect-game question when the
  player owns any perfect-aware item (Clown Shoes flips a No into a
  perfect at 50%), and a Level Up question driven by the character's
  level_up_condition. Crown re-rolls for bonus levels; item rewards use
  the existing RewardScreen.
- New items: clown_shoes.tres, crown.tres. Ironclad given level-up data.
- Excel items sheet: filled the Effect column for Clown Shoes and Crown.
- Tests for level-up stat application and item flag loading.
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10978" uniqueCount="3483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10980" uniqueCount="3485">
   <si>
     <t>Rogue</t>
   </si>
@@ -10516,6 +10516,12 @@
   </si>
   <si>
     <t>Gain +5 Speed this combat/event</t>
+  </si>
+  <si>
+    <t>perfect: verify Did you Perfect this game? =&gt; 50% to treat a non-perfect game as perfected</t>
+  </si>
+  <si>
+    <t>level_up: 50% chance to Level Up an additional time</t>
   </si>
 </sst>
 </file>
@@ -55566,6 +55572,9 @@
       <c r="D30" t="s">
         <v>1418</v>
       </c>
+      <c r="E30" t="s">
+        <v>3483</v>
+      </c>
       <c r="F30" t="s">
         <v>742</v>
       </c>
@@ -55594,6 +55603,9 @@
       </c>
       <c r="D31" t="s">
         <v>2851</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3484</v>
       </c>
       <c r="F31" t="s">
         <v>231</v>

</xml_diff>

<commit_message>
Add Empty Syringe and the Frozen/Molten/Toxic Eggs
Four data-driven items, each expressed as a declarative ItemData field so
the engine stays generic (no item-name matching):

- Empty Syringe (status_amplify): inflicting positive Bleed/Poison stacks
  on a non-player actor adds +1. Hooked in CombatActor.add_status, so it
  fires in every combat mode; never amplifies decay or the player's own
  buffs.
- Molten / Toxic / Frozen Egg (upgrade_card_types): auto-upgrade an
  Attack / Skill / Power card the moment it's added to the deck. Resolved
  in a new GameState.add_card_to_deck, which card rewards and shop
  purchases now route through (starting deck and weapon-granted cards stay
  direct).

Adds the two ItemData fields + helpers (GameState.status_amplify_bonus,
add_card_to_deck), the four .tres, the Effect column for each row in the
spreadsheet, and GUT coverage.
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -64703,6 +64703,11 @@
           <t>When Inflicting Bleed or Poison, Inflict +1 Bleed or Poison</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>status_amplify: +1 bleed, +1 poison (when inflicted on an enemy)</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>Mewgenics</t>
@@ -64844,6 +64849,11 @@
           <t>Whenever you add a Power card to your deck, Upgrade it</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>upgrade_card_types: power (auto-upgrade Power cards added to deck)</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>Slay the Spire</t>
@@ -65935,6 +65945,11 @@
           <t>Whenever you add an Attack card to your deck, Upgrade it</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>upgrade_card_types: attack (auto-upgrade Attack cards added to deck)</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>Slay the Spire</t>
@@ -67737,6 +67752,11 @@
       <c r="D105" t="inlineStr">
         <is>
           <t>Whenever you add a Skill card to your deck, Upgrade it</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>upgrade_card_types: skill (auto-upgrade Skill cards added to deck)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">

</xml_diff>

<commit_message>
Add Focus Crystal, Gremlin Horn, and Ice Cream
- Focus Crystal (attack_damage_bonus): the player's attacks gain flat per-hit
  damage by damage_type (+1 melee). Folded into Stats.damage_bonus for player
  sources only, so it applies in every combat mode.
- Gremlin Horn: declarative enemy_killed trigger -> gain_energy 1 + draw 1.
  Fires in all three modes (draw no-ops in strategy, which has no draw pile;
  gain_energy banks an empower charge there).
- Ice Cream (carries_leftover_energy): deckbuilder banks unspent energy at end
  of turn and pours it on next turn (can exceed max). Strategy analogue: a
  player turn that ends without an ability play banks an empower charge that
  stacks across turns. Action has no per-turn energy pool, so it's ignored.

Adds the new declarative ItemData fields + GameState helpers
(attack_damage_bonus, has_energy_carryover_item), the three .tres, the Effect
column for each spreadsheet row, and GUT coverage.
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -64802,6 +64802,11 @@
           <t>Melee Attacks deal +1 Dmg</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>attack_damage_bonus: {melee: 1} (player melee attacks deal +1)</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>Risk of Rain 2</t>
@@ -65042,6 +65047,11 @@
           <t>When an enemy dies, Gain +1 Energy and Draw 1 card</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>enemy_killed: gain_energy 1, draw 1</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>Slay the Spire</t>
@@ -65332,6 +65342,11 @@
       <c r="D53" t="inlineStr">
         <is>
           <t>When you end your turn with energy, gain that much energy on your next energy</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>carries_leftover_energy: true (deckbuilder carries leftover energy to next turn; strategy banks an empower charge on a turn the ability is skipped; action n/a)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">

</xml_diff>

<commit_message>
Fill in Effect column for the latest 8 items
https://claude.ai/code/session_01P22kqf7S6NuGXYFkb6Ng86
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -65000,6 +65000,11 @@
           <t>At the start of combat, gain +1 Brace</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>combat_started: +1 brace (self)</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>Super Auto Pets</t>
@@ -65240,6 +65245,11 @@
           <t>When you deal Dmg to an Enemy, 5% to Gain 1 Gold</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>attack_landed: 5% chance gain_gold 1</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>The Binding of Isaac</t>
@@ -66047,6 +66057,11 @@
           <t>When you kill an enemy, Gain +1 Brace</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>enemy_killed: +1 brace (self)</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>Mewgenics</t>
@@ -66146,6 +66161,11 @@
           <t>Gain +1 Field of View, get an extra option in the space choice</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>passive: +1 fov_bonus (an extra overworld portal option)</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>The Binding of Isaac</t>
@@ -66641,6 +66661,11 @@
           <t>Whenever you perfect a game (beat a game/combat without losing a run), Gain +5 Health</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>perfect: gain_hp 5</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
           <t>Haste</t>
@@ -66683,6 +66708,11 @@
           <t>Gain +1 Max Energy, but all enemies start with 1 Power</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>passive: +1 max_energy; enemy_spawned: +1 power (enemy)</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>Slay the Spire</t>
@@ -66730,6 +66760,11 @@
           <t>Whenever you take damage, Gain Temporary +3 Brace until end of this turn</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>damage_taken: +3 brace temp until end of turn (self)</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>Mewgenics</t>
@@ -66777,7 +66812,11 @@
           <t>33% chance to gain +1 Buffer each time you take damage</t>
         </is>
       </c>
-      <c r="E80" s="3" t="n"/>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>damage_taken: 33% chance +1 buffer (self)</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>Mewgenics</t>

</xml_diff>

<commit_message>
Fill in Effect column for Sacred Orb, Secret Technique Instructions, Shuriken, Snowball
https://claude.ai/code/session_01P22kqf7S6NuGXYFkb6Ng86
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -67307,6 +67307,11 @@
           <t>Whenever an item spawns, if it was Common, reroll it. If it was an Uncommon, there is a 25% chance to reroll it.</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>reroll_low_rarity: item rewards reroll Common picks (always) and Uncommon picks (25%)</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>The Binding of Isaac</t>
@@ -67354,6 +67359,11 @@
           <t>Whenever you perfect a game (beat a game/combat without losing a run), gain +1 Dash</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>perfect: gain_stat dash 1</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>Haste</t>
@@ -67401,6 +67411,11 @@
           <t>Every time you play 3 attacks in a single turn, Gain +1 Power</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>card_played if_type=attack: counter key=attacks_this_turn every=3 -&gt; +1 power (self)</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>Slay the Spire</t>
@@ -67446,6 +67461,11 @@
       <c r="D93" t="inlineStr">
         <is>
           <t>Whenever you would Gain permanent Intelligence, Gain +1 Intelligence</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>stat_gain_bonus: {intelligence: 1} (each permanent Intelligence gain grants +1 more)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">

</xml_diff>

<commit_message>
Flip items to sheet-generated; backport polished prose into the sheet
Backport all 89 hand-authored .tres descriptions (87 changed) and 6 reconciled
tag sets into the items sheet so nothing polished is lost, then regenerate every
data/items/*.tres from the sheet via generate_item_tres.py.

Verified semantically: parsing the pre-flip files and diffing field-by-field
against the regenerated output yields 0 differences (descriptions, tags,
source_game, effects, charge/use fields all preserved). The only on-disk change
is formatting — multi-line arrays collapse to single-line JSON.

https://claude.ai/code/session_01K7Djw7mZY2g18HUpffktir
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -66964,7 +66964,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gain +25 Max Health, but All Enemies start with +3 Health</t>
+          <t>Gain 25 Max HP, but all enemies spawn with +3 HP.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -67016,7 +67016,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +10 Block</t>
+          <t>At the start of combat, gain 10 Block.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -67068,7 +67068,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Add the Card "Bag o' Glitter" into your Deck. If you obtain something glittery at least one time, "Bag o' Glitter" Gains (+1/+2) Blind</t>
+          <t>Add the card "Bag o' Glitter" to your deck. If you obtain something glittery, it gains (+1/+2) Blind.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -67120,7 +67120,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gain +1 Speed</t>
+          <t>Gain 1 Speed.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -67172,7 +67172,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Add the Card "Barrel" into your Deck. If you obtain at least 1 fish, Gain (1/2) random fish</t>
+          <t>Add the card "Barrel" to your deck. If you obtained at least 1 fish, it gains (+1/+2) Dmg.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -67224,7 +67224,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +4 Block and +1 Bleed Thorns</t>
+          <t>At the start of combat, gain 4 Block and 1 Bleed Thorns.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -67239,7 +67239,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>wearable, mask</t>
+          <t>mask, trap</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -67276,7 +67276,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gain scaling +1 Strength per 20 max health </t>
+          <t>Gain +1 Strength per 20 Max HP.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -67291,7 +67291,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>wearable, ring</t>
+          <t>ring, scaling</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -67343,7 +67343,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>bird, devilish</t>
+          <t>head, bird</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -67380,7 +67380,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Add the Card "Blasma Pistol" into your Deck. If you open more than 10 chests, Gain (10/20) Gold</t>
+          <t>Add the card "Blasma Pistol" to your deck. If you opened more than 10 chests, gain (10/20) gold.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -67432,7 +67432,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Add the Card "Blood Magic" into your Deck. If you create or use a magic circle, "Blood Magic" Gains  (+1/+2/) Infuse</t>
+          <t>Add the card "Blood Magic" to your deck. If you created or used a magic circle, it gains (+1/+2) Infuse.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -67443,6 +67443,11 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Megabonk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>magic, blood</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -67479,7 +67484,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>At the start of combat, gain +2 Health</t>
+          <t>At the start of combat, gain 2 HP.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -67783,7 +67788,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gain +3 Luck and 18 Harvesting, but -3% Crit Chance</t>
+          <t>Gain +3 Luck and +18 Harvesting, but -3% Crit Chance.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -67835,7 +67840,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gain +5 Intelligence this combat/event</t>
+          <t>Gain +5 Intelligence this combat/event.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -67850,7 +67855,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>drug, pill, consumable</t>
+          <t>drug, pill, devilish</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -67887,7 +67892,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Your Strikes inflict Bruise</t>
+          <t>Your Strikes inflict Bruise.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -67898,6 +67903,11 @@
       <c r="F21" t="inlineStr">
         <is>
           <t>Mewgenics</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>offense</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -67934,7 +67944,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +3 Bleed Thorns and +1 Bleed</t>
+          <t>At the start of combat, gain 3 Bleed Thorns and 1 Bleed.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -67986,7 +67996,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +3 Thorns</t>
+          <t>At the start of combat, gain 3 Thorns.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -68038,7 +68048,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>At the end of combat, Gain +6 Health</t>
+          <t>At the end of combat, heal 6 HP.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -68085,7 +68095,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gain +1 Max Energy, but -2 Discovery</t>
+          <t>Gain +1 Max Energy, but -2 Discovery.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -68137,7 +68147,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Gain +3 Intelligence and +1 Regeneration, but -1 Speed</t>
+          <t>Gain +3 Intelligence and +1 Regeneration, but -1 Speed.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -68184,7 +68194,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Start the 3rd turn of combat with +18 Block</t>
+          <t>Start the 3rd turn of combat with 18 Block.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -68236,7 +68246,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>When you defeat an enemy, 50% chance to Heal +2 Health</t>
+          <t>When you defeat an enemy, 50% chance to heal 2 HP.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -68283,7 +68293,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Gain +5 Luck this combat/event</t>
+          <t>Gain +5 Luck this combat/event.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -68335,7 +68345,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Whenever you don't Perfect a game, (beat a game/combat without losing a run) 50% chance to treat it like you did</t>
+          <t>Whenever you don't Perfect a game (beat a game without losing a run), 50% chance to treat it like you did.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -68387,7 +68397,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>When Levelling Up, 50% chance to Level Up an additional time</t>
+          <t>When Levelling Up, 50% chance to Level Up an additional time.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -68439,7 +68449,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Gain +1 Reroll</t>
+          <t>Gain +1 Reroll.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -68590,7 +68600,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>When you play a power, deal Xx2 damage to each enemy where X is the amount of Curses you have</t>
+          <t>When you play a Power, deal Xx2 damage to each enemy, where X is the number of Curses you have.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -68684,7 +68694,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Gain +5 Charisma this combat/event</t>
+          <t>Gain +5 Charisma this combat/event.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -68736,7 +68746,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Your Weapon Attack Cards gain Replay 1</t>
+          <t>Your Weapon Attack Cards gain Replay 1.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -68788,7 +68798,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>At the start of each combat, Gain X Power where X is the amount of curses you have</t>
+          <t>At the start of each combat, gain X Power, where X is the number of Curses you have.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -68840,7 +68850,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>When Inflicting Bleed or Poison, Inflict +1 Bleed or Poison</t>
+          <t>When Inflicting Bleed or Poison, Inflict +1 Bleed or Poison.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -68939,7 +68949,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Melee Attacks deal +1 Dmg</t>
+          <t>Melee Attacks deal +1 Dmg.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -68991,7 +69001,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Whenever you add a Power card to your deck, Upgrade it</t>
+          <t>Whenever you add a Power card to your deck, Upgrade it.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -69043,7 +69053,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>At the start of combat, gain +1 Brace</t>
+          <t>At the start of combat, gain +1 Brace.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -69147,7 +69157,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Whenever you get rid of a Curse or Curse Card, gain one Chest</t>
+          <t>Whenever you get rid of a Curse or a Curse Card, gain one Chest.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -69199,7 +69209,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>When an enemy dies, Gain +1 Energy and Draw 1 card</t>
+          <t>When an enemy dies, Gain +1 Energy and Draw 1 card.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -69246,7 +69256,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Every 3 turns, Gain +1 energy</t>
+          <t>Every 3 turns, Gain +1 Energy.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -69298,7 +69308,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>When you deal Dmg to an Enemy, 5% to Gain 1 Gold</t>
+          <t>When you deal damage to an enemy, 5% chance to gain 1 Gold.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -69350,7 +69360,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Gain +12 Max Health</t>
+          <t>Gain 6 Max HP.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -69402,7 +69412,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +1 Buffer</t>
+          <t>At the start of combat, gain 1 Buffer.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -69454,7 +69464,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Start the 2nd turn of combat with +14 Block</t>
+          <t>Start the 2nd turn of combat with 14 Block.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -69506,7 +69516,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>When you end your turn with energy, gain that much energy on your next energy</t>
+          <t>Energy carries over between turns. (Strategy: skipping your ability banks an empower charge.)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -69558,7 +69568,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Your Strikes inflict Leeches</t>
+          <t>Your Strikes inflict Leeches.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -69610,7 +69620,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Gain 5 Gold. Whenever you spend 10 Gold, Gain +1 to a Random Stat</t>
+          <t>Gain 5 Gold. Whenever you spend 10 Gold, gain +1 to a random stat.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -69657,7 +69667,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>At the start of conflict, inflict +1 Leeches to all enemies. If you start combat above 50% health, lose 10 health</t>
+          <t>At the start of combat, inflict +1 Leeches to all enemies. If you start combat above 50% Health, lose 10 Health.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -69709,7 +69719,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Your Strikes Gain Heal 1</t>
+          <t>Your Strikes Gain Heal 1.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -69808,7 +69818,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Attacks deal 25% more Dmg to targets with lower Health</t>
+          <t>Attacks deal 25% more Dmg to targets with lower Health than you.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -69907,7 +69917,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Gain +2 Luck</t>
+          <t>Gain +2 Luck.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -69954,7 +69964,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Gain +8 Max Health and +8 Health</t>
+          <t>Gain 6 Max HP and 6 HP.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -70006,7 +70016,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Gain + 14 Max Health and +14 Health</t>
+          <t>Gain 14 Max HP and 14 HP.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -70058,7 +70068,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Whenever your Health is at 50% or below Max Health at the end of combat, gain +12 Health</t>
+          <t>If your Health is at 50% or below at the end of combat, gain +12 Health.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -70110,7 +70120,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>When you kill an enemy, Gain +1 Brace</t>
+          <t>When you kill an enemy, gain +1 Brace.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -70162,7 +70172,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Whenever you add an Attack card to your deck, Upgrade it</t>
+          <t>Whenever you add an Attack card to your deck, Upgrade it.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -70214,7 +70224,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Gain +1 Field of View, get an extra option in the space choice</t>
+          <t>Gain +1 Field of View (an extra portal option on the overworld).</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -70261,7 +70271,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>When you play a power, a random card in your hand becomes free to play this turn</t>
+          <t>When you play a Power, a random card becomes free this turn (deckbuilder: a hand card costs 0; strategy: another ability needs no play; action: cooldowns are slashed).</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -70313,7 +70323,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Every time you play 10 attacks, gain +1 Energy</t>
+          <t>Every time you play 10 Attacks, Gain +1 Energy.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -70365,7 +70375,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Gain +3 Dexterity</t>
+          <t>Gain +3 Dexterity.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -70417,7 +70427,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Gain 100 Gold</t>
+          <t>Gain 100 Gold.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -70469,7 +70479,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Every time you play 4 attacks in a single turn, Gain +4 Block</t>
+          <t>Every time you play 4 Attacks in a single turn, Gain +4 Block.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -70563,7 +70573,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Your Charisma is equal to your highest stat</t>
+          <t>Your Charisma is equal to your highest stat.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -70615,7 +70625,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Every 10th attack you play deals double damage</t>
+          <t>Every 10th Attack you play deals double damage.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -70662,7 +70672,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Gain +10 Block</t>
+          <t>Gain +10 Block. In combat it shields you; in an event it absorbs the next 10 damage.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -70714,7 +70724,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Whenever you perfect a game (beat a game/combat without losing a run), Gain +5 Health</t>
+          <t>Whenever you perfect a game (beat it without losing a run), gain +5 Health.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -70761,7 +70771,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Gain +1 Max Energy, but all enemies start with 1 Power</t>
+          <t>Gain +1 Max Energy, but all enemies start with 1 Power.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -70813,7 +70823,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Whenever you take damage, Gain Temporary +3 Brace until end of this turn</t>
+          <t>Whenever you take damage, gain a temporary +3 Brace until the end of the turn.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -70865,7 +70875,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>33% chance to gain +1 Buffer each time you take damage</t>
+          <t>Each time you take damage, 33% chance to gain +1 Buffer.</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -70964,7 +70974,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>At the start of combat, Gain +1 Regeneration</t>
+          <t>At the start of combat, gain 1 Regeneration.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -71016,7 +71026,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>At the start of combat, inflict Soul Link on 2 random enemies</t>
+          <t>At the start of combat, inflict Soul Link on 2 random enemies.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -71068,7 +71078,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>If the player would take lethal damage, negate that damage and destroy this item</t>
+          <t>If you would take lethal damage, negate that damage. Then this item is destroyed.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -71162,7 +71172,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>At the start of combat, Draw 2 Cards</t>
+          <t>At the start of combat, Draw 2 Cards.</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -71214,7 +71224,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Prevents your Strength, Dexterity, Intelligence, Charisma, FoV, Discovery, and Luck from falling below their highest values reached.</t>
+          <t>Your Strength, Dexterity, Intelligence, Charisma, FoV, Discovery, and Luck can never fall below the highest values they have reached.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -71266,7 +71276,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Gain +5 Strength this combat/event</t>
+          <t>Gain +5 Strength this combat/event.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -71360,7 +71370,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Whenever an item spawns, if it was Common, reroll it. If it was an Uncommon, there is a 25% chance to reroll it.</t>
+          <t>When item rewards appear, Common picks are always rerolled and Uncommon picks have a 25% chance to be rerolled.</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -71412,7 +71422,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Whenever you perfect a game (beat a game/combat without losing a run), gain +1 Dash</t>
+          <t>Whenever you perfect a game (beat it without losing a run), gain +1 Dash.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -71464,7 +71474,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Every time you play 3 attacks in a single turn, Gain +1 Power</t>
+          <t>Every time you play 3 Attacks in a single turn, Gain +1 Power.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -71516,7 +71526,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Whenever you would Gain permanent Intelligence, Gain +1 Intelligence</t>
+          <t>Whenever you would gain permanent Intelligence, gain +1 additional Intelligence.</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -71568,7 +71578,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Gain +5 Dexterity this combat/event</t>
+          <t>Gain +5 Dexterity this combat/event.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -71620,7 +71630,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Gain +6 Dexterity</t>
+          <t>Gain +6 Dexterity.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -71672,7 +71682,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Whenever you perfect a game (beat a game/combat without losing a run), Gain +10 Gold</t>
+          <t>Whenever you perfect a game (beat it without losing a run), gain 10 Gold.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -71766,7 +71776,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>At the end of turn 7, Deal 52 Damage to all enemies</t>
+          <t>At the end of turn 7, deal 52 damage to all enemies.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -71818,7 +71828,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Your Strikes Gain +3 Dmg</t>
+          <t>Your Strikes Gain +3 Dmg.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -71870,7 +71880,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>At the start of your turn, Gain +D12 Block</t>
+          <t>At the start of your turn, gain Block equal to a D12 roll (Luck helps as it normally does).</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -72100,7 +72110,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Whenever you add a Skill card to your deck, Upgrade it</t>
+          <t>Whenever you add a Skill card to your deck, Upgrade it.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -72199,7 +72209,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Gain +5 Speed this combat/event</t>
+          <t>Gain +5 Speed this combat/event.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -72251,7 +72261,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Gain +3 Strength</t>
+          <t>Gain 3 Strength.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -72340,7 +72350,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Gain +8 Max Health whenever you obtain a Curse</t>
+          <t>Gain +8 Max Health whenever you obtain a Curse.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -72439,7 +72449,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Upgrade 2 random Skills</t>
+          <t>Upgrade 2 random Skills.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -72533,7 +72543,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Upgrade 2 random Attacks</t>
+          <t>Upgrade 2 random Attacks.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -72679,7 +72689,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>50% Chance to Gain 1, 5, or 10 Gold</t>
+          <t>50% chance to gain 1, 5, or 10 gold. Luck biases the payout toward the bigger amounts.</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">

</xml_diff>

<commit_message>
Add Slimed status card to the cardsnew sheet
Adds the Slimed status card (Type Status, cost 1, Exhaust) to cardsnew so the
sheet is the source of truth for it. Round-trips exactly to the existing
hand-written data/cards/slimed.tres via generate_card_tres, so no .tres change
is needed; the slimes' add_card -> conjure:slimed now traces back to the sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019HSGEvHkFMWgKzoTWSoJKi
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -434,7 +434,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Table22" displayName="Table22" ref="A1:O55" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Table22" displayName="Table22" ref="A1:O56" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:O55"/>
   <sortState ref="A2:O53">
     <sortCondition ref="A33:A53"/>
@@ -31024,10 +31024,6 @@
           <t>effect_value</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -43065,7 +43061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -47137,6 +47133,81 @@
       <c r="O55" t="inlineStr">
         <is>
           <t>weapon</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Slimed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Exhaust.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Slimed</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Slay the Spire</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Exhaust</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cards: Slimed draws 1, add Beam (sweeping) card, generate Claw
Applies the cardsnew edits and regenerates the .tres the game loads:
- Slimed now draws 1 card then Exhausts (StS2), instead of a dead Exhaust.
- Adds 'Beam' (the old Sweeping Beam, renamed): Deal 6 Dmg Ranged Cleave,
  Draw 1 Card, on a new sweep_beam attack archetype.
- Claw (already in the sheet) now has its generated claw.tres.

sweep_beam archetype, added to the generator + both attack libraries:
- Action: a full-length beam that pans left-to-right across a wide arc,
  striking each enemy as the beam crosses its angle (reuses the swing
  timing) with a beam-line visual + swept-area wedge.
- Strategy: a wide (spread) full-range line, so it reads as one large
  sweeping attack at beam range rather than a thin single-target zap.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PEXjREUNUsHKms5JjeEH5N
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -43061,7 +43061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -47157,12 +47157,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Exhaust.</t>
+          <t>Draw 1 Card. Exhaust.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draw:1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -47208,6 +47208,79 @@
       <c r="O56" t="inlineStr">
         <is>
           <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Beam</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Deal 6 Dmg Ranged Cleave. Draw 1 Card.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>dmg:6:ranged:cleave; draw:1</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Deal 9 Dmg Ranged Cleave. Draw 1 Card.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>dmg:9:ranged:cleave; draw:1</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>sweep_beam</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>SweepingBeam</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Slay the Spire</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>defect, offense, draw</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Encounters sheet: fill Effect + Requirement Effect columns
Author the machine-readable Effect and Requirement Effect strings for the
7 overworld encounters (Deal with the Devil, P Mart / Trorc shopkeepers,
Teleporter, Divine Teleporter, Challenge Rift, Angel Room), matching the
existing scrolls-sheet DSL (space-delimited tokens, semicolon-separated
clauses) so a future generate_encounter_tres.py parses them like the
scroll generator.

Edited the .xlsx surgically (only xl/worksheets/sheet6.xml) to preserve
sharedStrings and relationship formatting the project's hand-rolled XML
readers depend on.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvJffBNminYJ8BPMmaCW2p
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -78144,6 +78144,11 @@
       <c r="D2" t="s">
         <v>5439</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">offer_items evil 3 any ; per_item lose_hp_pct by_rarity ; per_item add_curse 1</t>
+        </is>
+      </c>
       <c r="F2" t="s">
         <v>5426</v>
       </c>
@@ -78152,6 +78157,11 @@
       </c>
       <c r="H2" t="s">
         <v>5455</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">last_game.curses_triggered &gt;= 1</t>
+        </is>
       </c>
       <c r="J2" t="s">
         <v>5422</v>
@@ -78170,6 +78180,11 @@
       <c r="D3" t="s">
         <v>5436</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shop food pill</t>
+        </is>
+      </c>
       <c r="F3" t="s">
         <v>5431</v>
       </c>
@@ -78193,6 +78208,11 @@
       <c r="D4" t="s">
         <v>5437</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shop military discount=20</t>
+        </is>
+      </c>
       <c r="F4" t="s">
         <v>5438</v>
       </c>
@@ -78216,6 +78236,11 @@
       <c r="D5" t="s">
         <v>5445</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">combat action elite ; teleport nearby</t>
+        </is>
+      </c>
       <c r="F5" t="s">
         <v>2715</v>
       </c>
@@ -78239,6 +78264,11 @@
       <c r="D6" t="s">
         <v>5446</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">combat action elite ; teleport choose nearby previous</t>
+        </is>
+      </c>
       <c r="F6" t="s">
         <v>2715</v>
       </c>
@@ -78262,6 +78292,11 @@
       <c r="D7" t="s">
         <v>5449</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">challenge action unconnected attempts=3 ; win gain_gold 50 ; win gain_chest ; lose add_curse 1</t>
+        </is>
+      </c>
       <c r="F7" t="s">
         <v>2715</v>
       </c>
@@ -78285,6 +78320,11 @@
       <c r="D8" t="s">
         <v>5452</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">offer_items holy 3 one</t>
+        </is>
+      </c>
       <c r="F8" t="s">
         <v>2715</v>
       </c>
@@ -78293,6 +78333,11 @@
       </c>
       <c r="H8" t="s">
         <v>5451</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">last_game.curses_held &gt;= 2 and last_game.curses_triggered == 0</t>
+        </is>
       </c>
       <c r="J8" t="s">
         <v>5453</v>

</xml_diff>

<commit_message>
Challenge Rift: reward up front on commit, curse on failure
Restructure the Challenge encounter: committing to play a random unconnected
game now grants its reward (gold + item chest) immediately, then you must beat
it within N attempts or take a random curse. Renames the challenge effect
buckets win/lose -> reward/fail across the encounters sheet, generator, .tres,
modal flow, and test.

Also add a SessionStart hook (.claude/) for Claude Code on the web: installs the
Godot 4.6 engine + openpyxl and warms the import cache so the vendored GUT suite
(godot --headless -s addons/gut/gut_cmdln.gd) runs in fresh remote containers.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvJffBNminYJ8BPMmaCW2p
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -78289,12 +78289,14 @@
       <c r="C7" t="s">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
-        <v>5449</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decide to play a Random Action Game not connected on the map to claim 50 Gold and a Chest up front. Then beat it within 3 attempts — fail and gain a Random Curse.</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">challenge action unconnected attempts=3 ; win gain_gold 50 ; win gain_chest ; lose add_curse 1</t>
+          <t xml:space="preserve">challenge action unconnected attempts=3 ; reward gain_gold 50 ; reward gain_chest ; fail add_curse 1</t>
         </is>
       </c>
       <c r="F7" t="s">

</xml_diff>

<commit_message>
Challenge Rift: reward up front on commit, curse on failure (#111)
</commit_message>
<xml_diff>
--- a/tools/Roguelikes.xlsx
+++ b/tools/Roguelikes.xlsx
@@ -78144,6 +78144,11 @@
       <c r="D2" t="s">
         <v>5439</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">offer_items evil 3 any ; per_item lose_hp_pct by_rarity ; per_item add_curse 1</t>
+        </is>
+      </c>
       <c r="F2" t="s">
         <v>5426</v>
       </c>
@@ -78152,6 +78157,11 @@
       </c>
       <c r="H2" t="s">
         <v>5455</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">last_game.curses_triggered &gt;= 1</t>
+        </is>
       </c>
       <c r="J2" t="s">
         <v>5422</v>
@@ -78170,6 +78180,11 @@
       <c r="D3" t="s">
         <v>5436</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shop food pill</t>
+        </is>
+      </c>
       <c r="F3" t="s">
         <v>5431</v>
       </c>
@@ -78193,6 +78208,11 @@
       <c r="D4" t="s">
         <v>5437</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shop military discount=20</t>
+        </is>
+      </c>
       <c r="F4" t="s">
         <v>5438</v>
       </c>
@@ -78216,6 +78236,11 @@
       <c r="D5" t="s">
         <v>5445</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">combat action elite ; teleport nearby</t>
+        </is>
+      </c>
       <c r="F5" t="s">
         <v>2715</v>
       </c>
@@ -78239,6 +78264,11 @@
       <c r="D6" t="s">
         <v>5446</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">combat action elite ; teleport choose nearby previous</t>
+        </is>
+      </c>
       <c r="F6" t="s">
         <v>2715</v>
       </c>
@@ -78259,8 +78289,15 @@
       <c r="C7" t="s">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
-        <v>5449</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decide to play a Random Action Game not connected on the map to claim 50 Gold and a Chest up front. Then beat it within 3 attempts — fail and gain a Random Curse.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">challenge action unconnected attempts=3 ; reward gain_gold 50 ; reward gain_chest ; fail add_curse 1</t>
+        </is>
       </c>
       <c r="F7" t="s">
         <v>2715</v>
@@ -78285,6 +78322,11 @@
       <c r="D8" t="s">
         <v>5452</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">offer_items holy 3 one</t>
+        </is>
+      </c>
       <c r="F8" t="s">
         <v>2715</v>
       </c>
@@ -78293,6 +78335,11 @@
       </c>
       <c r="H8" t="s">
         <v>5451</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">last_game.curses_held &gt;= 2 and last_game.curses_triggered == 0</t>
+        </is>
       </c>
       <c r="J8" t="s">
         <v>5453</v>

</xml_diff>